<commit_message>
cambio comparacion manualvsalgoritmo y porcentaje de llenado a lo largo del contenedor
</commit_message>
<xml_diff>
--- a/plantilla_deliveries.xlsx
+++ b/plantilla_deliveries.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deliveries" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -422,6 +423,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,6 +457,11 @@
           <t>Alto (ft)</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -475,6 +482,9 @@
       <c r="F2" t="n">
         <v>5.96</v>
       </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -495,6 +505,9 @@
       <c r="F3" t="n">
         <v>3.61</v>
       </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -514,6 +527,130 @@
       </c>
       <c r="F4" t="n">
         <v>3.68</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TR-620</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1003</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TR-450</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1004</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TR-620</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1005</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Instrucciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Esta misma plantilla se usa en dos lugares de la app:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1) Subir deliveries para que el algoritmo calcule el mejor acomodo: la columna 'Caja' no es necesaria, puede dejarse vacía.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2) Subir tu propio acomodo manual para comparar contra el algoritmo: la columna 'Caja' es obligatoria y debe indicar a qué caja (1, 2, 3...) va cada delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>'Bulto extra': deja vacío si no aplica, o escribe 'y' por cada bulto extra (y = 1, yy = 2, yyy = 3...).</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>